<commit_message>
Sources de vérité : note EN 13053 (PDC) + date Bibliothèque à jour
- DONNEES_PDC : note de convention en A4 — ΔP finale = min(ΔP init + ADD ;
  3×ΔP init), ADD +50 Pa (Coarse) / +100 Pa (ePM). Ligne NETFIBRE r9 confirmée
  (poly 14·v²+1,8·v+8, ΔP nom 42 Pa).
- Bibliothèque : « Mise à jour » → 22/06/2026 ; ligne NETFIBRE r6 finalisée.
- (CLAUDE.md du projet mis à jour hors dépôt : NETFIBRE ✅, règles EN 13053
  et température média, rangement _Archive.)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/DONNEES_PDC_Netair.xlsx
+++ b/fiches-techniques/DONNEES_PDC_Netair.xlsx
@@ -599,6 +599,13 @@
         <v>3400</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ΔP finale recommandée (EN 13053) = min(ΔP initiale + ADD ; 3 × ΔP initiale) — ADD = +50 Pa (Coarse) / +100 Pa (ePM10·ePM2,5·ePM1). Idem calculateur ; jamais les valeurs absolues Titanair.</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="30" customHeight="1" s="22">
       <c r="A5" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
NETCEL V AZUR : courbe H13 corrigée (axe débit comprimé de 20 %) — DONNEES_PDC réaligné
Erreur détectée par PA sur la fiche source PDF (TITAPAK V-GD 592 H13) : notre
extraction du cache Excel portait les bonnes ΔP aux mauvais débits (400-2400 au
lieu de 500-3000). Polynôme réajusté (20,3525·v²+95,8058·v−14,70, R²=0,999) dans
le JSON ET dans DONNEES_PDC_Netair.xlsx l.58 (la source de vérité devait suivre
immédiatement — demande PA) ; ΔP@nominal E10 l.57 recalée sur le nominal 3000.
Au passage (passe v1.1 en cours, validée étape par étape) : descriptif PA, plage
E10→H14 (H14 sur devis), points clés PA, tableau technique et dimensions refaits
(3 formats, nominaux 3000/2500/1500, en-tête EN 1822 via nouvelle clé
dims_entete_eff), surface 24 m² retirée par prudence, boutique restreinte aux
classes EPA/HEPA — le F8 490×592 à 12 € (cellule Excel erronée) n'est plus
commandable ; relevé au centime identique sur les classes conservées.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fiches-techniques/DONNEES_PDC_Netair.xlsx
+++ b/fiches-techniques/DONNEES_PDC_Netair.xlsx
@@ -4859,11 +4859,11 @@
       <c r="S57" s="40" t="n"/>
       <c r="T57" s="41" t="n"/>
       <c r="U57" s="41" t="n">
-        <v>134</v>
+        <v>176</v>
       </c>
       <c r="V57" s="36" t="inlineStr">
         <is>
-          <t>Mode HEPA (ΔP finale=2×init). Cache Excel TITAPAK V GD E10 : débit [1000-3500] → ΔP [50,79,108,140,176,212].</t>
+          <t>Mode HEPA (ΔP finale=2×init). Cache Excel TITAPAK V GD E10 : débit [1000-3500] → ΔP [50,79,108,140,176,212]. Nominal fiche 3000 m³/h (02/08/2026).</t>
         </is>
       </c>
     </row>
@@ -4909,10 +4909,10 @@
       <c r="M58" s="37" t="n"/>
       <c r="N58" s="37" t="n"/>
       <c r="O58" s="38" t="n">
-        <v>31.8</v>
+        <v>20.3525</v>
       </c>
       <c r="P58" s="38" t="n">
-        <v>119.76</v>
+        <v>95.8058</v>
       </c>
       <c r="Q58" s="38" t="n">
         <v>-14.7</v>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="V58" s="36" t="inlineStr">
         <is>
-          <t>Mode HEPA (ΔP finale=2×init). Cache Excel TITAPAK V-GD 592 H13 (24 m²) : débit [400-2400] → ΔP [25,75,131,188,250,331]. Extrapolé &gt;2400.</t>
+          <t>Mode HEPA (ΔP finale=2×init). Cache Excel TITAPAK V-GD 592 H13 (24 m²) : débit [500-3000] → ΔP [25,75,131,188,250,331]. ✅ AXE DÉBIT CORRIGÉ 02/08/2026 (fiche source PDF ; l’extraction du cache comprimait l’axe de 20 % : 400-2400. Erreur détectée PA). Nominal fiche 3000 m³/h.</t>
         </is>
       </c>
     </row>

</xml_diff>